<commit_message>
Bug is Solved (Bias) And Forword version of Mul is Added
</commit_message>
<xml_diff>
--- a/Mul/testcases.xlsx
+++ b/Mul/testcases.xlsx
@@ -508,17 +508,17 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1072223893</v>
+        <v>2628454108</v>
       </c>
       <c r="B2" t="n">
-        <v>57373178</v>
+        <v>3447962165</v>
       </c>
       <c r="C2" s="1">
         <f>(A2*B2)</f>
         <v/>
       </c>
       <c r="D2" t="n">
-        <v>6.151689226894195e+16</v>
+        <v>1.622042995763552e+19</v>
       </c>
       <c r="E2" s="1">
         <f>IF(C2=D2,"PASS","FAIL")</f>
@@ -527,17 +527,17 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2638978784</v>
+        <v>370883053</v>
       </c>
       <c r="B3" t="n">
-        <v>946765817</v>
+        <v>1980184530</v>
       </c>
       <c r="C3" s="1">
         <f>(A3*B3)</f>
         <v/>
       </c>
       <c r="D3" t="n">
-        <v>1.660848365614863e+19</v>
+        <v>7.344168839897701e+17</v>
       </c>
       <c r="E3" s="1">
         <f>IF(C3=D3,"PASS","FAIL")</f>
@@ -546,17 +546,17 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>4024414125</v>
+        <v>1785718112</v>
       </c>
       <c r="B4" t="n">
-        <v>96459939</v>
+        <v>643729083</v>
       </c>
       <c r="C4" s="1">
         <f>(A4*B4)</f>
         <v/>
       </c>
       <c r="D4" t="n">
-        <v>1.842064653133864e+19</v>
+        <v>1.149518682734251e+18</v>
       </c>
       <c r="E4" s="1">
         <f>IF(C4=D4,"PASS","FAIL")</f>
@@ -565,17 +565,17 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2620452512</v>
+        <v>3322948819</v>
       </c>
       <c r="B5" t="n">
-        <v>1546006468</v>
+        <v>2589362627</v>
       </c>
       <c r="C5" s="1">
         <f>(A5*B5)</f>
         <v/>
       </c>
       <c r="D5" t="n">
-        <v>1.700719571679354e+19</v>
+        <v>1.277910705317512e+19</v>
       </c>
       <c r="E5" s="1">
         <f>IF(C5=D5,"PASS","FAIL")</f>
@@ -584,17 +584,17 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1086028490</v>
+        <v>4043102011</v>
       </c>
       <c r="B6" t="n">
-        <v>1137958253</v>
+        <v>1402554823</v>
       </c>
       <c r="C6" s="1">
         <f>(A6*B6)</f>
         <v/>
       </c>
       <c r="D6" t="n">
-        <v>1.235855083188628e+18</v>
+        <v>5.670672225409049e+18</v>
       </c>
       <c r="E6" s="1">
         <f>IF(C6=D6,"PASS","FAIL")</f>
@@ -603,17 +603,17 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>2417893842</v>
+        <v>2440949844</v>
       </c>
       <c r="B7" t="n">
-        <v>1845433272</v>
+        <v>3098049558</v>
       </c>
       <c r="C7" s="1">
         <f>(A7*B7)</f>
         <v/>
       </c>
       <c r="D7" t="n">
-        <v>6.682587686508261e+16</v>
+        <v>1.552512790785762e+19</v>
       </c>
       <c r="E7" s="1">
         <f>IF(C7=D7,"PASS","FAIL")</f>
@@ -622,17 +622,17 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>1085435575</v>
+        <v>264183520</v>
       </c>
       <c r="B8" t="n">
-        <v>1818120401</v>
+        <v>2998324667</v>
       </c>
       <c r="C8" s="1">
         <f>(A8*B8)</f>
         <v/>
       </c>
       <c r="D8" t="n">
-        <v>1.969230438228006e+18</v>
+        <v>1.810419245979828e+19</v>
       </c>
       <c r="E8" s="1">
         <f>IF(C8=D8,"PASS","FAIL")</f>
@@ -641,17 +641,17 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2417941760</v>
+        <v>2161607139</v>
       </c>
       <c r="B9" t="n">
-        <v>2625506353</v>
+        <v>770482502</v>
       </c>
       <c r="C9" s="1">
         <f>(A9*B9)</f>
         <v/>
       </c>
       <c r="D9" t="n">
-        <v>1.813933330478742e+19</v>
+        <v>1.665480476797782e+18</v>
       </c>
       <c r="E9" s="1">
         <f>IF(C9=D9,"PASS","FAIL")</f>
@@ -660,17 +660,17 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>3583433102</v>
+        <v>1958923201</v>
       </c>
       <c r="B10" t="n">
-        <v>1115557817</v>
+        <v>2866151433</v>
       </c>
       <c r="C10" s="1">
         <f>(A10*B10)</f>
         <v/>
       </c>
       <c r="D10" t="n">
-        <v>1.765298654153006e+19</v>
+        <v>1.564780352972201e+19</v>
       </c>
       <c r="E10" s="1">
         <f>IF(C10=D10,"PASS","FAIL")</f>
@@ -679,17 +679,17 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>693933272</v>
+        <v>1337579634</v>
       </c>
       <c r="B11" t="n">
-        <v>4158709776</v>
+        <v>1009721063</v>
       </c>
       <c r="C11" s="1">
         <f>(A11*B11)</f>
         <v/>
       </c>
       <c r="D11" t="n">
-        <v>1.835219044702135e+19</v>
+        <v>1.350582329889631e+18</v>
       </c>
       <c r="E11" s="1">
         <f>IF(C11=D11,"PASS","FAIL")</f>
@@ -698,17 +698,17 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>2061971956</v>
+        <v>1871068076</v>
       </c>
       <c r="B12" t="n">
-        <v>1963746469</v>
+        <v>4115250038</v>
       </c>
       <c r="C12" s="1">
         <f>(A12*B12)</f>
         <v/>
       </c>
       <c r="D12" t="n">
-        <v>1.781213348595122e+19</v>
+        <v>1.81104808495595e+19</v>
       </c>
       <c r="E12" s="1">
         <f>IF(C12=D12,"PASS","FAIL")</f>
@@ -717,17 +717,17 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>2708365418</v>
+        <v>535749757</v>
       </c>
       <c r="B13" t="n">
-        <v>1085749554</v>
+        <v>1266631383</v>
       </c>
       <c r="C13" s="1">
         <f>(A13*B13)</f>
         <v/>
       </c>
       <c r="D13" t="n">
-        <v>1.672521328986085e+19</v>
+        <v>6.785974556508239e+17</v>
       </c>
       <c r="E13" s="1">
         <f>IF(C13=D13,"PASS","FAIL")</f>
@@ -736,17 +736,17 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>4251405088</v>
+        <v>2612882355</v>
       </c>
       <c r="B14" t="n">
-        <v>3588311436</v>
+        <v>172421658</v>
       </c>
       <c r="C14" s="1">
         <f>(A14*B14)</f>
         <v/>
       </c>
       <c r="D14" t="n">
-        <v>3.078348955773888e+16</v>
+        <v>4.505175078080446e+17</v>
       </c>
       <c r="E14" s="1">
         <f>IF(C14=D14,"PASS","FAIL")</f>
@@ -755,17 +755,17 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>1002746256</v>
+        <v>1058020422</v>
       </c>
       <c r="B15" t="n">
-        <v>66179757</v>
+        <v>2805158369</v>
       </c>
       <c r="C15" s="1">
         <f>(A15*B15)</f>
         <v/>
       </c>
       <c r="D15" t="n">
-        <v>6.636150355473979e+16</v>
+        <v>1.687049580406564e+19</v>
       </c>
       <c r="E15" s="1">
         <f>IF(C15=D15,"PASS","FAIL")</f>
@@ -774,17 +774,17 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>406187326</v>
+        <v>3046565422</v>
       </c>
       <c r="B16" t="n">
-        <v>1296037387</v>
+        <v>798588420</v>
       </c>
       <c r="C16" s="1">
         <f>(A16*B16)</f>
         <v/>
       </c>
       <c r="D16" t="n">
-        <v>5.264339606215572e+17</v>
+        <v>2.432951866781613e+18</v>
       </c>
       <c r="E16" s="1">
         <f>IF(C16=D16,"PASS","FAIL")</f>
@@ -793,17 +793,17 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>2312232302</v>
+        <v>1500441784</v>
       </c>
       <c r="B17" t="n">
-        <v>3344794655</v>
+        <v>438548579</v>
       </c>
       <c r="C17" s="1">
         <f>(A17*B17)</f>
         <v/>
       </c>
       <c r="D17" t="n">
-        <v>2.176885696383191e+18</v>
+        <v>6.580166122454249e+17</v>
       </c>
       <c r="E17" s="1">
         <f>IF(C17=D17,"PASS","FAIL")</f>
@@ -812,17 +812,17 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>3109826291</v>
+        <v>3007788651</v>
       </c>
       <c r="B18" t="n">
-        <v>870128075</v>
+        <v>2885212351</v>
       </c>
       <c r="C18" s="1">
         <f>(A18*B18)</f>
         <v/>
       </c>
       <c r="D18" t="n">
-        <v>1.742002321205271e+19</v>
+        <v>1.420649914944742e+19</v>
       </c>
       <c r="E18" s="1">
         <f>IF(C18=D18,"PASS","FAIL")</f>
@@ -831,17 +831,17 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>2939675424</v>
+        <v>2920836478</v>
       </c>
       <c r="B19" t="n">
-        <v>2844628151</v>
+        <v>1335967237</v>
       </c>
       <c r="C19" s="1">
         <f>(A19*B19)</f>
         <v/>
       </c>
       <c r="D19" t="n">
-        <v>1.731656797651066e+18</v>
+        <v>3.902141839242471e+18</v>
       </c>
       <c r="E19" s="1">
         <f>IF(C19=D19,"PASS","FAIL")</f>
@@ -850,17 +850,17 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>2189753963</v>
+        <v>3529713890</v>
       </c>
       <c r="B20" t="n">
-        <v>2010728332</v>
+        <v>3599469853</v>
       </c>
       <c r="C20" s="1">
         <f>(A20*B20)</f>
         <v/>
       </c>
       <c r="D20" t="n">
-        <v>1.796410869300369e+19</v>
+        <v>1.599183708869297e+19</v>
       </c>
       <c r="E20" s="1">
         <f>IF(C20=D20,"PASS","FAIL")</f>
@@ -869,17 +869,17 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>2596115415</v>
+        <v>2406935055</v>
       </c>
       <c r="B21" t="n">
-        <v>3848279041</v>
+        <v>3154133048</v>
       </c>
       <c r="C21" s="1">
         <f>(A21*B21)</f>
         <v/>
       </c>
       <c r="D21" t="n">
-        <v>1.806619055021217e+19</v>
+        <v>1.570083013025379e+19</v>
       </c>
       <c r="E21" s="1">
         <f>IF(C21=D21,"PASS","FAIL")</f>
@@ -888,17 +888,17 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>2754753037</v>
+        <v>3137179931</v>
       </c>
       <c r="B22" t="n">
-        <v>1300924667</v>
+        <v>1247534820</v>
       </c>
       <c r="C22" s="1">
         <f>(A22*B22)</f>
         <v/>
       </c>
       <c r="D22" t="n">
-        <v>1.649700978044908e+19</v>
+        <v>3.913741200527697e+18</v>
       </c>
       <c r="E22" s="1">
         <f>IF(C22=D22,"PASS","FAIL")</f>
@@ -907,17 +907,17 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>699305904</v>
+        <v>1778000736</v>
       </c>
       <c r="B23" t="n">
-        <v>591003993</v>
+        <v>1717082165</v>
       </c>
       <c r="C23" s="1">
         <f>(A23*B23)</f>
         <v/>
       </c>
       <c r="D23" t="n">
-        <v>4.132925815924747e+17</v>
+        <v>3.052973353142473e+18</v>
       </c>
       <c r="E23" s="1">
         <f>IF(C23=D23,"PASS","FAIL")</f>
@@ -926,17 +926,17 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>1699732133</v>
+        <v>4200175189</v>
       </c>
       <c r="B24" t="n">
-        <v>3183558508</v>
+        <v>3057895054</v>
       </c>
       <c r="C24" s="1">
         <f>(A24*B24)</f>
         <v/>
       </c>
       <c r="D24" t="n">
-        <v>1.648558897493153e+19</v>
+        <v>1.325082393586055e+19</v>
       </c>
       <c r="E24" s="1">
         <f>IF(C24=D24,"PASS","FAIL")</f>
@@ -945,17 +945,17 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>3736360531</v>
+        <v>1693860206</v>
       </c>
       <c r="B25" t="n">
-        <v>729405604</v>
+        <v>1772595117</v>
       </c>
       <c r="C25" s="1">
         <f>(A25*B25)</f>
         <v/>
       </c>
       <c r="D25" t="n">
-        <v>1.803929316888624e+19</v>
+        <v>3.002528330036214e+18</v>
       </c>
       <c r="E25" s="1">
         <f>IF(C25=D25,"PASS","FAIL")</f>
@@ -964,17 +964,17 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>1674001895</v>
+        <v>966762532</v>
       </c>
       <c r="B26" t="n">
-        <v>183589385</v>
+        <v>3966969740</v>
       </c>
       <c r="C26" s="1">
         <f>(A26*B26)</f>
         <v/>
       </c>
       <c r="D26" t="n">
-        <v>3.073125028973371e+17</v>
+        <v>1.812964832598118e+19</v>
       </c>
       <c r="E26" s="1">
         <f>IF(C26=D26,"PASS","FAIL")</f>
@@ -983,17 +983,17 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>555553233</v>
+        <v>3703318403</v>
       </c>
       <c r="B27" t="n">
-        <v>1394456658</v>
+        <v>3503268653</v>
       </c>
       <c r="C27" s="1">
         <f>(A27*B27)</f>
         <v/>
       </c>
       <c r="D27" t="n">
-        <v>7.746949046302753e+17</v>
+        <v>1.551483191945752e+19</v>
       </c>
       <c r="E27" s="1">
         <f>IF(C27=D27,"PASS","FAIL")</f>
@@ -1002,17 +1002,17 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>3776215055</v>
+        <v>1512693939</v>
       </c>
       <c r="B28" t="n">
-        <v>1335395798</v>
+        <v>1409410050</v>
       </c>
       <c r="C28" s="1">
         <f>(A28*B28)</f>
         <v/>
       </c>
       <c r="D28" t="n">
-        <v>1.775400451087507e+19</v>
+        <v>2.132006040200687e+18</v>
       </c>
       <c r="E28" s="1">
         <f>IF(C28=D28,"PASS","FAIL")</f>
@@ -1021,17 +1021,17 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>1557832347</v>
+        <v>2888720276</v>
       </c>
       <c r="B29" t="n">
-        <v>3611318275</v>
+        <v>3307779373</v>
       </c>
       <c r="C29" s="1">
         <f>(A29*B29)</f>
         <v/>
       </c>
       <c r="D29" t="n">
-        <v>1.709348994450962e+19</v>
+        <v>1.559503430431712e+19</v>
       </c>
       <c r="E29" s="1">
         <f>IF(C29=D29,"PASS","FAIL")</f>
@@ -1040,17 +1040,17 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>3169448428</v>
+        <v>961597736</v>
       </c>
       <c r="B30" t="n">
-        <v>3556836982</v>
+        <v>1174313225</v>
       </c>
       <c r="C30" s="1">
         <f>(A30*B30)</f>
         <v/>
       </c>
       <c r="D30" t="n">
-        <v>8.307796083346665e+17</v>
+        <v>1.129216938514859e+18</v>
       </c>
       <c r="E30" s="1">
         <f>IF(C30=D30,"PASS","FAIL")</f>
@@ -1059,17 +1059,17 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>1065213357</v>
+        <v>3178908820</v>
       </c>
       <c r="B31" t="n">
-        <v>2036873097</v>
+        <v>2135694755</v>
       </c>
       <c r="C31" s="1">
         <f>(A31*B31)</f>
         <v/>
       </c>
       <c r="D31" t="n">
-        <v>2.169704429438357e+18</v>
+        <v>6.78917889349724e+18</v>
       </c>
       <c r="E31" s="1">
         <f>IF(C31=D31,"PASS","FAIL")</f>
@@ -1078,17 +1078,17 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>285887973</v>
+        <v>2542048245</v>
       </c>
       <c r="B32" t="n">
-        <v>1002839850</v>
+        <v>1866720848</v>
       </c>
       <c r="C32" s="1">
         <f>(A32*B32)</f>
         <v/>
       </c>
       <c r="D32" t="n">
-        <v>2.866998519601241e+17</v>
+        <v>4.745294455563312e+18</v>
       </c>
       <c r="E32" s="1">
         <f>IF(C32=D32,"PASS","FAIL")</f>
@@ -1097,17 +1097,17 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>3185471475</v>
+        <v>1085925707</v>
       </c>
       <c r="B33" t="n">
-        <v>3272308056</v>
+        <v>1127704520</v>
       </c>
       <c r="C33" s="1">
         <f>(A33*B33)</f>
         <v/>
       </c>
       <c r="D33" t="n">
-        <v>1.134636204626644e+18</v>
+        <v>1.224603328168096e+18</v>
       </c>
       <c r="E33" s="1">
         <f>IF(C33=D33,"PASS","FAIL")</f>
@@ -1116,17 +1116,17 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>1625418540</v>
+        <v>912023322</v>
       </c>
       <c r="B34" t="n">
-        <v>654602234</v>
+        <v>369648488</v>
       </c>
       <c r="C34" s="1">
         <f>(A34*B34)</f>
         <v/>
       </c>
       <c r="D34" t="n">
-        <v>1.928623371474943e+18</v>
+        <v>3.371280419980371e+17</v>
       </c>
       <c r="E34" s="1">
         <f>IF(C34=D34,"PASS","FAIL")</f>
@@ -1135,17 +1135,17 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>4123114671</v>
+        <v>753347139</v>
       </c>
       <c r="B35" t="n">
-        <v>1417182185</v>
+        <v>333678091</v>
       </c>
       <c r="C35" s="1">
         <f>(A35*B35)</f>
         <v/>
       </c>
       <c r="D35" t="n">
-        <v>1.820319759511407e+19</v>
+        <v>2.513754352018316e+17</v>
       </c>
       <c r="E35" s="1">
         <f>IF(C35=D35,"PASS","FAIL")</f>
@@ -1154,17 +1154,17 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>4274861758</v>
+        <v>3165307292</v>
       </c>
       <c r="B36" t="n">
-        <v>2481587330</v>
+        <v>3528319507</v>
       </c>
       <c r="C36" s="1">
         <f>(A36*B36)</f>
         <v/>
       </c>
       <c r="D36" t="n">
-        <v>3.645897981485171e+16</v>
+        <v>1.602006823679217e+19</v>
       </c>
       <c r="E36" s="1">
         <f>IF(C36=D36,"PASS","FAIL")</f>
@@ -1173,17 +1173,17 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>3416029267</v>
+        <v>2703597327</v>
       </c>
       <c r="B37" t="n">
-        <v>325975705</v>
+        <v>710420778</v>
       </c>
       <c r="C37" s="1">
         <f>(A37*B37)</f>
         <v/>
       </c>
       <c r="D37" t="n">
-        <v>1.816023163005497e+19</v>
+        <v>1.92069171644606e+18</v>
       </c>
       <c r="E37" s="1">
         <f>IF(C37=D37,"PASS","FAIL")</f>
@@ -1192,17 +1192,17 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>402858240</v>
+        <v>2043138762</v>
       </c>
       <c r="B38" t="n">
-        <v>1120267376</v>
+        <v>3037128164</v>
       </c>
       <c r="C38" s="1">
         <f>(A38*B38)</f>
         <v/>
       </c>
       <c r="D38" t="n">
-        <v>4.513089434247782e+17</v>
+        <v>1.587680418675992e+19</v>
       </c>
       <c r="E38" s="1">
         <f>IF(C38=D38,"PASS","FAIL")</f>
@@ -1211,17 +1211,17 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>279828106</v>
+        <v>1235000588</v>
       </c>
       <c r="B39" t="n">
-        <v>2417445848</v>
+        <v>2978227632</v>
       </c>
       <c r="C39" s="1">
         <f>(A39*B39)</f>
         <v/>
       </c>
       <c r="D39" t="n">
-        <v>1.792136080294133e+19</v>
+        <v>1.682056981442663e+19</v>
       </c>
       <c r="E39" s="1">
         <f>IF(C39=D39,"PASS","FAIL")</f>
@@ -1230,17 +1230,17 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>395863133</v>
+        <v>2275977129</v>
       </c>
       <c r="B40" t="n">
-        <v>3248943353</v>
+        <v>2132407794</v>
       </c>
       <c r="C40" s="1">
         <f>(A40*B40)</f>
         <v/>
       </c>
       <c r="D40" t="n">
-        <v>1.803266175844056e+19</v>
+        <v>4.853311368845344e+18</v>
       </c>
       <c r="E40" s="1">
         <f>IF(C40=D40,"PASS","FAIL")</f>
@@ -1249,17 +1249,17 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>2401808811</v>
+        <v>2281565507</v>
       </c>
       <c r="B41" t="n">
-        <v>2336070747</v>
+        <v>1526168949</v>
       </c>
       <c r="C41" s="1">
         <f>(A41*B41)</f>
         <v/>
       </c>
       <c r="D41" t="n">
-        <v>1.840847955667205e+19</v>
+        <v>3.482054431892842e+18</v>
       </c>
       <c r="E41" s="1">
         <f>IF(C41=D41,"PASS","FAIL")</f>
@@ -1268,17 +1268,17 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>306624848</v>
+        <v>2410554930</v>
       </c>
       <c r="B42" t="n">
-        <v>464270505</v>
+        <v>3086358103</v>
       </c>
       <c r="C42" s="1">
         <f>(A42*B42)</f>
         <v/>
       </c>
       <c r="D42" t="n">
-        <v>1.423568730265082e+17</v>
+        <v>1.553332522508008e+19</v>
       </c>
       <c r="E42" s="1">
         <f>IF(C42=D42,"PASS","FAIL")</f>
@@ -1287,17 +1287,17 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>4146259396</v>
+        <v>2659930382</v>
       </c>
       <c r="B43" t="n">
-        <v>1369345307</v>
+        <v>2291414936</v>
       </c>
       <c r="C43" s="1">
         <f>(A43*B43)</f>
         <v/>
       </c>
       <c r="D43" t="n">
-        <v>1.824311160873073e+19</v>
+        <v>1.311743427941775e+19</v>
       </c>
       <c r="E43" s="1">
         <f>IF(C43=D43,"PASS","FAIL")</f>
@@ -1306,17 +1306,17 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>2729552624</v>
+        <v>117708755</v>
       </c>
       <c r="B44" t="n">
-        <v>4212143434</v>
+        <v>1233567220</v>
       </c>
       <c r="C44" s="1">
         <f>(A44*B44)</f>
         <v/>
       </c>
       <c r="D44" t="n">
-        <v>1.29653684471536e+17</v>
+        <v>1.452016616750111e+17</v>
       </c>
       <c r="E44" s="1">
         <f>IF(C44=D44,"PASS","FAIL")</f>
@@ -1325,17 +1325,17 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>4056321040</v>
+        <v>199633434</v>
       </c>
       <c r="B45" t="n">
-        <v>747462322</v>
+        <v>3692468369</v>
       </c>
       <c r="C45" s="1">
         <f>(A45*B45)</f>
         <v/>
       </c>
       <c r="D45" t="n">
-        <v>1.826836498906318e+19</v>
+        <v>1.832646514393123e+19</v>
       </c>
       <c r="E45" s="1">
         <f>IF(C45=D45,"PASS","FAIL")</f>
@@ -1344,17 +1344,17 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>3966995004</v>
+        <v>303049630</v>
       </c>
       <c r="B46" t="n">
-        <v>1991422518</v>
+        <v>3385621218</v>
       </c>
       <c r="C46" s="1">
         <f>(A46*B46)</f>
         <v/>
       </c>
       <c r="D46" t="n">
-        <v>1.779361266614068e+19</v>
+        <v>1.81711670812297e+19</v>
       </c>
       <c r="E46" s="1">
         <f>IF(C46=D46,"PASS","FAIL")</f>
@@ -1363,17 +1363,17 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>3067015803</v>
+        <v>931703555</v>
       </c>
       <c r="B47" t="n">
-        <v>313379448</v>
+        <v>3348886056</v>
       </c>
       <c r="C47" s="1">
         <f>(A47*B47)</f>
         <v/>
       </c>
       <c r="D47" t="n">
-        <v>1.806220994582556e+19</v>
+        <v>1.756527681908274e+19</v>
       </c>
       <c r="E47" s="1">
         <f>IF(C47=D47,"PASS","FAIL")</f>
@@ -1382,17 +1382,17 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>3206236224</v>
+        <v>1526203245</v>
       </c>
       <c r="B48" t="n">
-        <v>510052151</v>
+        <v>1650412897</v>
       </c>
       <c r="C48" s="1">
         <f>(A48*B48)</f>
         <v/>
       </c>
       <c r="D48" t="n">
-        <v>1.789143444857542e+19</v>
+        <v>2.518865518991251e+18</v>
       </c>
       <c r="E48" s="1">
         <f>IF(C48=D48,"PASS","FAIL")</f>
@@ -1401,17 +1401,17 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>4169611057</v>
+        <v>830022128</v>
       </c>
       <c r="B49" t="n">
-        <v>506427602</v>
+        <v>3177325439</v>
       </c>
       <c r="C49" s="1">
         <f>(A49*B49)</f>
         <v/>
       </c>
       <c r="D49" t="n">
-        <v>1.838326021419704e+19</v>
+        <v>1.751907660122054e+19</v>
       </c>
       <c r="E49" s="1">
         <f>IF(C49=D49,"PASS","FAIL")</f>
@@ -1420,17 +1420,17 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>3502574973</v>
+        <v>3614017476</v>
       </c>
       <c r="B50" t="n">
-        <v>728139293</v>
+        <v>1889398428</v>
       </c>
       <c r="C50" s="1">
         <f>(A50*B50)</f>
         <v/>
       </c>
       <c r="D50" t="n">
-        <v>1.78697720878617e+19</v>
+        <v>6.828318937918928e+18</v>
       </c>
       <c r="E50" s="1">
         <f>IF(C50=D50,"PASS","FAIL")</f>
@@ -1439,17 +1439,17 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>2533707271</v>
+        <v>1543836711</v>
       </c>
       <c r="B51" t="n">
-        <v>2222720574</v>
+        <v>2024375597</v>
       </c>
       <c r="C51" s="1">
         <f>(A51*B51)</f>
         <v/>
       </c>
       <c r="D51" t="n">
-        <v>1.750284106142745e+19</v>
+        <v>3.125305363501142e+18</v>
       </c>
       <c r="E51" s="1">
         <f>IF(C51=D51,"PASS","FAIL")</f>

</xml_diff>